<commit_message>
implementing the material search page
</commit_message>
<xml_diff>
--- a/creative-block/src/app/search/materials/MaterialDatabase.xlsx
+++ b/creative-block/src/app/search/materials/MaterialDatabase.xlsx
@@ -1,16 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="88" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9589DDCB-CCE5-46F0-9B5C-9276FC51549E}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Windows\System32\Team25_CreativeBlock\creative-block\src\app\search\materials\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD52479-F707-43EE-8734-C6527F43668D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yarn Entries" sheetId="1" r:id="rId1"/>
-    <sheet name="Fabric Entries" sheetId="2" r:id="rId2"/>
-    <sheet name="Thread Entries" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -33,103 +36,58 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
-  <si>
-    <t>Yarn Entry Associated User</t>
-  </si>
-  <si>
-    <t>Yarn Name</t>
-  </si>
-  <si>
-    <t>Yarn Image</t>
-  </si>
-  <si>
-    <t>Yarn Color</t>
-  </si>
-  <si>
-    <t>Yarn Amount Number</t>
-  </si>
-  <si>
-    <t>Yarn Amount Unit</t>
-  </si>
-  <si>
-    <t>Yarn Weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yarn Fiber Type </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Yarn Entry Date Added</t>
-  </si>
-  <si>
-    <t>Fabric Entry Associated User</t>
-  </si>
-  <si>
-    <t>Fabric Name</t>
-  </si>
-  <si>
-    <t>Fabric Image</t>
-  </si>
-  <si>
-    <t>Fabric Color</t>
-  </si>
-  <si>
-    <t>Fabric Length Number</t>
-  </si>
-  <si>
-    <t>Fabric Length Unit</t>
-  </si>
-  <si>
-    <t>Fabric Width Number</t>
-  </si>
-  <si>
-    <t>Fabric Width Unit</t>
-  </si>
-  <si>
-    <t>Fabric Pattern Description</t>
-  </si>
-  <si>
-    <t>Fabric Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabric Entry Date Added </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thread Entry Associated User </t>
-  </si>
-  <si>
-    <t>Thread Name</t>
-  </si>
-  <si>
-    <t>Thread Image</t>
-  </si>
-  <si>
-    <t>Thread Color</t>
-  </si>
-  <si>
-    <t>Thread Amount Number</t>
-  </si>
-  <si>
-    <t>Thread Amount Unit</t>
-  </si>
-  <si>
-    <t>Thread Tex</t>
-  </si>
-  <si>
-    <t>Thread Denier</t>
-  </si>
-  <si>
-    <t>Thread Weight</t>
-  </si>
-  <si>
-    <t>Thread Entry Date Added</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Date Added</t>
+  </si>
+  <si>
+    <t>Used In</t>
+  </si>
+  <si>
+    <t>Yarn</t>
+  </si>
+  <si>
+    <t>Bernat</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>meowmeowmeow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bernat Blanket Extra Faded Blues </t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/I/81OIFCd-D3L._AC_SX569_.jpg</t>
+  </si>
+  <si>
+    <t>Material Name</t>
+  </si>
+  <si>
+    <t>Material Image</t>
+  </si>
+  <si>
+    <t>Material Type</t>
+  </si>
+  <si>
+    <t>Material Brand</t>
+  </si>
+  <si>
+    <t>Material Color</t>
+  </si>
+  <si>
+    <t>Material Id</t>
+  </si>
+  <si>
+    <t>#Used In</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,8 +116,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -178,9 +137,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -218,7 +177,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -324,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,7 +425,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -474,182 +433,105 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AA3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.1796875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="13" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.81640625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="13" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="23.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46118</v>
+      </c>
+      <c r="E2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="1"/>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD60FE2E-C988-4033-BE95-F2AFBD3485A6}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75007D69-D1A8-4D0D-9ECF-94405BF2941F}">
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>